<commit_message>
Harden Zhizunbao import and add price overrides
</commit_message>
<xml_diff>
--- a/imports/881133521557/product-input.xlsx
+++ b/imports/881133521557/product-input.xlsx
@@ -488,7 +488,7 @@
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>test002</t>
+          <t>test004</t>
         </is>
       </c>
     </row>
@@ -567,10 +567,14 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
         <v>198</v>
@@ -595,13 +599,17 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="4">
@@ -623,13 +631,17 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="5">
@@ -651,13 +663,17 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="6">
@@ -679,13 +695,17 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="7">
@@ -707,13 +727,17 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="8">
@@ -735,13 +759,17 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="9">
@@ -763,10 +791,14 @@
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
         <v>198</v>
@@ -791,13 +823,17 @@
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="11">
@@ -819,13 +855,17 @@
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="n">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="12">
@@ -847,13 +887,17 @@
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="13">
@@ -875,13 +919,17 @@
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="14">
@@ -903,13 +951,17 @@
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="15">
@@ -931,10 +983,14 @@
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="n">
         <v>198</v>
@@ -959,13 +1015,17 @@
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="17">
@@ -987,13 +1047,17 @@
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="18">
@@ -1015,13 +1079,17 @@
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="19">
@@ -1043,13 +1111,17 @@
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="20">
@@ -1071,13 +1143,17 @@
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="21">
@@ -1099,13 +1175,17 @@
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="22">
@@ -1127,13 +1207,17 @@
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="23">
@@ -1155,13 +1239,17 @@
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="24">
@@ -1183,13 +1271,17 @@
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="25">
@@ -1211,13 +1303,17 @@
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="26">
@@ -1239,13 +1335,17 @@
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="27">
@@ -1267,13 +1367,17 @@
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="28">
@@ -1295,13 +1399,17 @@
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="29">
@@ -1323,13 +1431,17 @@
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="30">
@@ -1351,13 +1463,17 @@
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="31">
@@ -1379,13 +1495,17 @@
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="32">
@@ -1407,13 +1527,17 @@
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="33">
@@ -1435,13 +1559,17 @@
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="n">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="34">
@@ -1463,13 +1591,17 @@
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="35">
@@ -1491,13 +1623,17 @@
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="36">
@@ -1519,13 +1655,17 @@
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="37">
@@ -1547,10 +1687,14 @@
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="n">
         <v>198</v>
@@ -1575,13 +1719,17 @@
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="39">
@@ -1603,13 +1751,17 @@
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="40">
@@ -1631,13 +1783,17 @@
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="41">
@@ -1659,13 +1815,17 @@
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="42">
@@ -1687,13 +1847,17 @@
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="43">
@@ -1715,13 +1879,17 @@
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="44">
@@ -1743,13 +1911,17 @@
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="45">
@@ -1771,13 +1943,17 @@
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="46">
@@ -1799,13 +1975,17 @@
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="47">
@@ -1827,13 +2007,17 @@
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="48">
@@ -1855,13 +2039,17 @@
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="49">
@@ -1883,13 +2071,17 @@
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="50">
@@ -1911,13 +2103,17 @@
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="51">
@@ -1939,13 +2135,17 @@
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="52">
@@ -1967,13 +2167,17 @@
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="53">
@@ -1995,13 +2199,17 @@
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="54">
@@ -2023,13 +2231,17 @@
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="55">
@@ -2051,13 +2263,17 @@
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr">
         <is>
-          <t>146.64</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr"/>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refine multi-shop draft flow and skip detail image uploads
</commit_message>
<xml_diff>
--- a/imports/881133521557/product-input.xlsx
+++ b/imports/881133521557/product-input.xlsx
@@ -488,7 +488,7 @@
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>test004</t>
+          <t>test001</t>
         </is>
       </c>
     </row>
@@ -567,7 +567,7 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -577,7 +577,7 @@
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="3">
@@ -599,7 +599,7 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -609,7 +609,7 @@
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="4">
@@ -631,7 +631,7 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -641,7 +641,7 @@
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="5">
@@ -663,7 +663,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -673,7 +673,7 @@
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="6">
@@ -695,7 +695,7 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -705,7 +705,7 @@
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="7">
@@ -727,7 +727,7 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -737,7 +737,7 @@
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="8">
@@ -759,7 +759,7 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -769,7 +769,7 @@
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="9">
@@ -791,7 +791,7 @@
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -801,7 +801,7 @@
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="10">
@@ -823,7 +823,7 @@
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -833,7 +833,7 @@
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="11">
@@ -855,7 +855,7 @@
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -865,7 +865,7 @@
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="12">
@@ -887,7 +887,7 @@
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -897,7 +897,7 @@
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="13">
@@ -919,7 +919,7 @@
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -929,7 +929,7 @@
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="14">
@@ -951,7 +951,7 @@
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="15">
@@ -983,7 +983,7 @@
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -993,7 +993,7 @@
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="16">
@@ -1015,7 +1015,7 @@
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1025,7 +1025,7 @@
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="17">
@@ -1047,7 +1047,7 @@
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="18">
@@ -1079,7 +1079,7 @@
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1089,7 +1089,7 @@
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="19">
@@ -1111,7 +1111,7 @@
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1121,7 +1121,7 @@
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="20">
@@ -1143,7 +1143,7 @@
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1153,7 +1153,7 @@
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="21">
@@ -1175,7 +1175,7 @@
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="22">
@@ -1207,7 +1207,7 @@
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="23">
@@ -1239,7 +1239,7 @@
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1249,7 +1249,7 @@
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="24">
@@ -1271,7 +1271,7 @@
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1281,7 +1281,7 @@
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="25">
@@ -1303,7 +1303,7 @@
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1313,7 +1313,7 @@
       </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="26">
@@ -1335,7 +1335,7 @@
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="27">
@@ -1367,7 +1367,7 @@
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="28">
@@ -1399,7 +1399,7 @@
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="29">
@@ -1431,7 +1431,7 @@
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="30">
@@ -1463,7 +1463,7 @@
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1473,7 +1473,7 @@
       </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="31">
@@ -1495,7 +1495,7 @@
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="32">
@@ -1527,7 +1527,7 @@
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1537,7 +1537,7 @@
       </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="33">
@@ -1559,7 +1559,7 @@
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1569,7 +1569,7 @@
       </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="34">
@@ -1591,7 +1591,7 @@
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1601,7 +1601,7 @@
       </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="35">
@@ -1623,7 +1623,7 @@
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="36">
@@ -1655,7 +1655,7 @@
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="37">
@@ -1687,7 +1687,7 @@
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1697,7 +1697,7 @@
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="38">
@@ -1719,7 +1719,7 @@
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -1729,7 +1729,7 @@
       </c>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="39">
@@ -1751,7 +1751,7 @@
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -1761,7 +1761,7 @@
       </c>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="40">
@@ -1783,7 +1783,7 @@
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -1793,7 +1793,7 @@
       </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="41">
@@ -1815,7 +1815,7 @@
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -1825,7 +1825,7 @@
       </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="42">
@@ -1847,7 +1847,7 @@
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -1857,7 +1857,7 @@
       </c>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="43">
@@ -1879,7 +1879,7 @@
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -1889,7 +1889,7 @@
       </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="44">
@@ -1911,7 +1911,7 @@
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -1921,7 +1921,7 @@
       </c>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="45">
@@ -1943,7 +1943,7 @@
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -1953,7 +1953,7 @@
       </c>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="46">
@@ -1975,7 +1975,7 @@
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -1985,7 +1985,7 @@
       </c>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="47">
@@ -2007,7 +2007,7 @@
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2017,7 +2017,7 @@
       </c>
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="48">
@@ -2039,7 +2039,7 @@
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2049,7 +2049,7 @@
       </c>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="49">
@@ -2071,7 +2071,7 @@
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2081,7 +2081,7 @@
       </c>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="50">
@@ -2103,7 +2103,7 @@
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2113,7 +2113,7 @@
       </c>
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="51">
@@ -2135,7 +2135,7 @@
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2145,7 +2145,7 @@
       </c>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="52">
@@ -2167,7 +2167,7 @@
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -2177,7 +2177,7 @@
       </c>
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="53">
@@ -2199,7 +2199,7 @@
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -2209,7 +2209,7 @@
       </c>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="54">
@@ -2231,7 +2231,7 @@
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -2241,7 +2241,7 @@
       </c>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
     <row r="55">
@@ -2263,7 +2263,7 @@
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>146.64</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -2273,7 +2273,7 @@
       </c>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="n">
-        <v>198</v>
+        <v>500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Handle recommended category popups and manual checks
</commit_message>
<xml_diff>
--- a/imports/881133521557/product-input.xlsx
+++ b/imports/881133521557/product-input.xlsx
@@ -488,7 +488,7 @@
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>test001</t>
+          <t>006</t>
         </is>
       </c>
     </row>
@@ -567,7 +567,7 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -577,7 +577,7 @@
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="3">
@@ -599,7 +599,7 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -609,7 +609,7 @@
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="4">
@@ -631,7 +631,7 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -641,7 +641,7 @@
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="5">
@@ -663,7 +663,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -673,7 +673,7 @@
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="6">
@@ -695,7 +695,7 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -705,7 +705,7 @@
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="7">
@@ -727,7 +727,7 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -737,7 +737,7 @@
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="8">
@@ -759,7 +759,7 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -769,7 +769,7 @@
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="9">
@@ -791,7 +791,7 @@
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -801,7 +801,7 @@
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="10">
@@ -823,7 +823,7 @@
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -833,7 +833,7 @@
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="11">
@@ -855,7 +855,7 @@
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -865,7 +865,7 @@
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="12">
@@ -887,7 +887,7 @@
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -897,7 +897,7 @@
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="13">
@@ -919,7 +919,7 @@
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -929,7 +929,7 @@
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="14">
@@ -951,7 +951,7 @@
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="15">
@@ -983,7 +983,7 @@
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -993,7 +993,7 @@
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="16">
@@ -1015,7 +1015,7 @@
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1025,7 +1025,7 @@
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="17">
@@ -1047,7 +1047,7 @@
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="18">
@@ -1079,7 +1079,7 @@
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1089,7 +1089,7 @@
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="19">
@@ -1111,7 +1111,7 @@
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1121,7 +1121,7 @@
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="20">
@@ -1143,7 +1143,7 @@
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1153,7 +1153,7 @@
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="21">
@@ -1175,7 +1175,7 @@
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="22">
@@ -1207,7 +1207,7 @@
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="23">
@@ -1239,7 +1239,7 @@
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1249,7 +1249,7 @@
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="24">
@@ -1271,7 +1271,7 @@
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1281,7 +1281,7 @@
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="25">
@@ -1303,7 +1303,7 @@
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1313,7 +1313,7 @@
       </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="26">
@@ -1335,7 +1335,7 @@
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="27">
@@ -1367,7 +1367,7 @@
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="28">
@@ -1399,7 +1399,7 @@
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="29">
@@ -1431,7 +1431,7 @@
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="30">
@@ -1463,7 +1463,7 @@
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1473,7 +1473,7 @@
       </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="31">
@@ -1495,7 +1495,7 @@
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="32">
@@ -1527,7 +1527,7 @@
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1537,7 +1537,7 @@
       </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="33">
@@ -1559,7 +1559,7 @@
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1569,7 +1569,7 @@
       </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="34">
@@ -1591,7 +1591,7 @@
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1601,7 +1601,7 @@
       </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="35">
@@ -1623,7 +1623,7 @@
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="36">
@@ -1655,7 +1655,7 @@
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="37">
@@ -1687,7 +1687,7 @@
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1697,7 +1697,7 @@
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="38">
@@ -1719,7 +1719,7 @@
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -1729,7 +1729,7 @@
       </c>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="39">
@@ -1751,7 +1751,7 @@
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -1761,7 +1761,7 @@
       </c>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="40">
@@ -1783,7 +1783,7 @@
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -1793,7 +1793,7 @@
       </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="41">
@@ -1815,7 +1815,7 @@
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -1825,7 +1825,7 @@
       </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="42">
@@ -1847,7 +1847,7 @@
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -1857,7 +1857,7 @@
       </c>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="43">
@@ -1879,7 +1879,7 @@
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -1889,7 +1889,7 @@
       </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="44">
@@ -1911,7 +1911,7 @@
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -1921,7 +1921,7 @@
       </c>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="45">
@@ -1943,7 +1943,7 @@
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -1953,7 +1953,7 @@
       </c>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="46">
@@ -1975,7 +1975,7 @@
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -1985,7 +1985,7 @@
       </c>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="47">
@@ -2007,7 +2007,7 @@
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2017,7 +2017,7 @@
       </c>
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="48">
@@ -2039,7 +2039,7 @@
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2049,7 +2049,7 @@
       </c>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="49">
@@ -2071,7 +2071,7 @@
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2081,7 +2081,7 @@
       </c>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="50">
@@ -2103,7 +2103,7 @@
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2113,7 +2113,7 @@
       </c>
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="51">
@@ -2135,7 +2135,7 @@
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2145,7 +2145,7 @@
       </c>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="52">
@@ -2167,7 +2167,7 @@
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -2177,7 +2177,7 @@
       </c>
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="53">
@@ -2199,7 +2199,7 @@
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -2209,7 +2209,7 @@
       </c>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="54">
@@ -2231,7 +2231,7 @@
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -2241,7 +2241,7 @@
       </c>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
     <row r="55">
@@ -2263,7 +2263,7 @@
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr">
         <is>
-          <t>146.64</t>
+          <t>146</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -2273,7 +2273,7 @@
       </c>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="n">
-        <v>500</v>
+        <v>199</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update product input workbook
</commit_message>
<xml_diff>
--- a/imports/881133521557/product-input.xlsx
+++ b/imports/881133521557/product-input.xlsx
@@ -577,7 +577,7 @@
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3">
@@ -609,7 +609,7 @@
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4">
@@ -641,7 +641,7 @@
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5">
@@ -673,7 +673,7 @@
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6">
@@ -705,7 +705,7 @@
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7">
@@ -737,7 +737,7 @@
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8">
@@ -769,7 +769,7 @@
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9">
@@ -801,7 +801,7 @@
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10">
@@ -833,7 +833,7 @@
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11">
@@ -865,7 +865,7 @@
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12">
@@ -897,7 +897,7 @@
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13">
@@ -929,7 +929,7 @@
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14">
@@ -961,7 +961,7 @@
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15">
@@ -993,7 +993,7 @@
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16">
@@ -1025,7 +1025,7 @@
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="17">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="18">
@@ -1089,7 +1089,7 @@
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="19">
@@ -1121,7 +1121,7 @@
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="20">
@@ -1153,7 +1153,7 @@
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="21">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="22">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="23">
@@ -1249,7 +1249,7 @@
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="24">
@@ -1281,7 +1281,7 @@
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="25">
@@ -1313,7 +1313,7 @@
       </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="26">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="27">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="28">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="29">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="30">
@@ -1473,7 +1473,7 @@
       </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="31">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="32">
@@ -1537,7 +1537,7 @@
       </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="33">
@@ -1569,7 +1569,7 @@
       </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="34">
@@ -1601,7 +1601,7 @@
       </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="35">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="36">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="37">
@@ -1697,7 +1697,7 @@
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="38">
@@ -1729,7 +1729,7 @@
       </c>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="39">
@@ -1761,7 +1761,7 @@
       </c>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="40">
@@ -1793,7 +1793,7 @@
       </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="41">
@@ -1825,7 +1825,7 @@
       </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="42">
@@ -1857,7 +1857,7 @@
       </c>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="43">
@@ -1889,7 +1889,7 @@
       </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="44">
@@ -1921,7 +1921,7 @@
       </c>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="45">
@@ -1953,7 +1953,7 @@
       </c>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="46">
@@ -1985,7 +1985,7 @@
       </c>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="47">
@@ -2017,7 +2017,7 @@
       </c>
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="48">
@@ -2049,7 +2049,7 @@
       </c>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="49">
@@ -2081,7 +2081,7 @@
       </c>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="50">
@@ -2113,7 +2113,7 @@
       </c>
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="51">
@@ -2145,7 +2145,7 @@
       </c>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="52">
@@ -2177,7 +2177,7 @@
       </c>
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="53">
@@ -2209,7 +2209,7 @@
       </c>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="54">
@@ -2241,7 +2241,7 @@
       </c>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
     <row r="55">
@@ -2273,7 +2273,7 @@
       </c>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="n">
-        <v>199</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>